<commit_message>
Update H1 titles: add rows 163-182
Claude-Session: https://claude.ai/code/session_01XSXZy4TLsyYfdEs2SnHeNG
</commit_message>
<xml_diff>
--- a/Appliance_parts_batch_1_H1_titles.xlsx
+++ b/Appliance_parts_batch_1_H1_titles.xlsx
@@ -5123,44 +5123,64 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="3" t="inlineStr">
+      <c r="A163" t="inlineStr">
         <is>
           <t>/products/danby-890011174</t>
         </is>
       </c>
-      <c r="B163" s="3" t="inlineStr">
+      <c r="B163" t="inlineStr">
         <is>
           <t>Danby</t>
         </is>
       </c>
-      <c r="C163" s="3" t="inlineStr"/>
-      <c r="D163" s="3" t="inlineStr">
-        <is>
-          <t>Not processed yet</t>
-        </is>
-      </c>
-      <c r="E163" s="3" t="inlineStr"/>
-      <c r="F163" s="3" t="inlineStr"/>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Danby Refrigerator Wire Freezer Shelf - 890011174</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr"/>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>genuinereplacementparts, encompass</t>
+        </is>
+      </c>
     </row>
     <row r="164">
-      <c r="A164" s="3" t="inlineStr">
+      <c r="A164" t="inlineStr">
         <is>
           <t>/products/danby-dar044a6bsldb</t>
         </is>
       </c>
-      <c r="B164" s="3" t="inlineStr">
+      <c r="B164" t="inlineStr">
         <is>
           <t>Danby</t>
         </is>
       </c>
-      <c r="C164" s="3" t="inlineStr"/>
-      <c r="D164" s="3" t="inlineStr">
-        <is>
-          <t>Not processed yet</t>
-        </is>
-      </c>
-      <c r="E164" s="3" t="inlineStr"/>
-      <c r="F164" s="3" t="inlineStr"/>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Danby 4.4 Cu. Ft. Outdoor Compact Refrigerator Stainless Steel - DAR044A6BSLDB</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Model number - whole appliance</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>SERP (townappliance, walmart, energystar - as DAR044A6BSLDBO)</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
@@ -5183,24 +5203,32 @@
       <c r="F165" s="3" t="inlineStr"/>
     </row>
     <row r="166">
-      <c r="A166" s="3" t="inlineStr">
+      <c r="A166" t="inlineStr">
         <is>
           <t>/products/goodman-zp29k5e-pfv-130</t>
         </is>
       </c>
-      <c r="B166" s="3" t="inlineStr">
+      <c r="B166" t="inlineStr">
         <is>
           <t>Goodman</t>
         </is>
       </c>
-      <c r="C166" s="3" t="inlineStr"/>
-      <c r="D166" s="3" t="inlineStr">
-        <is>
-          <t>Not processed yet</t>
-        </is>
-      </c>
-      <c r="E166" s="3" t="inlineStr"/>
-      <c r="F166" s="3" t="inlineStr"/>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Goodman HVAC Copeland 2.5 Ton R410A Scroll Compressor - ZP29K5E-PFV-130</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>SERP (ebay, technicalhotandcoldparts)</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="3" t="inlineStr">
@@ -5243,104 +5271,148 @@
       <c r="F168" s="3" t="inlineStr"/>
     </row>
     <row r="169">
-      <c r="A169" s="3" t="inlineStr">
+      <c r="A169" t="inlineStr">
         <is>
           <t>/products/kenmore-30120-0030100-00</t>
         </is>
       </c>
-      <c r="B169" s="3" t="inlineStr">
+      <c r="B169" t="inlineStr">
         <is>
           <t>Kenmore</t>
         </is>
       </c>
-      <c r="C169" s="3" t="inlineStr"/>
-      <c r="D169" s="3" t="inlineStr">
-        <is>
-          <t>Not processed yet</t>
-        </is>
-      </c>
-      <c r="E169" s="3" t="inlineStr"/>
-      <c r="F169" s="3" t="inlineStr"/>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Kenmore Refrigerator Evaporator Fan Motor Assembly - 30120-0030100-00</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr"/>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>searspartsdirect, genuinereplacementparts, shopjimmy, encompass</t>
+        </is>
+      </c>
     </row>
     <row r="170">
-      <c r="A170" s="3" t="inlineStr">
+      <c r="A170" t="inlineStr">
         <is>
           <t>/products/kenmore-3017837600</t>
         </is>
       </c>
-      <c r="B170" s="3" t="inlineStr">
+      <c r="B170" t="inlineStr">
         <is>
           <t>Kenmore</t>
         </is>
       </c>
-      <c r="C170" s="3" t="inlineStr"/>
-      <c r="D170" s="3" t="inlineStr">
-        <is>
-          <t>Not processed yet</t>
-        </is>
-      </c>
-      <c r="E170" s="3" t="inlineStr"/>
-      <c r="F170" s="3" t="inlineStr"/>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Kenmore Refrigerator Shelf Assembly - 3017837600</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr"/>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>encompass, searspartsdirect</t>
+        </is>
+      </c>
     </row>
     <row r="171">
-      <c r="A171" s="3" t="inlineStr">
+      <c r="A171" t="inlineStr">
         <is>
           <t>/products/lokring-appliance-a20160019</t>
         </is>
       </c>
-      <c r="B171" s="3" t="inlineStr">
+      <c r="B171" t="inlineStr">
         <is>
           <t>Lokring</t>
         </is>
       </c>
-      <c r="C171" s="3" t="inlineStr"/>
-      <c r="D171" s="3" t="inlineStr">
-        <is>
-          <t>Not processed yet</t>
-        </is>
-      </c>
-      <c r="E171" s="3" t="inlineStr"/>
-      <c r="F171" s="3" t="inlineStr"/>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Lokring Appliance LG Repair Kit - A20160019</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr"/>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>reliableparts, partadvantage, genuinereplacementparts</t>
+        </is>
+      </c>
     </row>
     <row r="172">
-      <c r="A172" s="3" t="inlineStr">
+      <c r="A172" t="inlineStr">
         <is>
           <t>/products/lokring-appliance-l14000166</t>
         </is>
       </c>
-      <c r="B172" s="3" t="inlineStr">
+      <c r="B172" t="inlineStr">
         <is>
           <t>Lokring</t>
         </is>
       </c>
-      <c r="C172" s="3" t="inlineStr"/>
-      <c r="D172" s="3" t="inlineStr">
-        <is>
-          <t>Not processed yet</t>
-        </is>
-      </c>
-      <c r="E172" s="3" t="inlineStr"/>
-      <c r="F172" s="3" t="inlineStr"/>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Lokring Appliance LRSZ 120 Degree Tube Cutter - L14000166</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr"/>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>reliableparts, encompass, partadvantage, genuinereplacementparts</t>
+        </is>
+      </c>
     </row>
     <row r="173">
-      <c r="A173" s="3" t="inlineStr">
+      <c r="A173" t="inlineStr">
         <is>
           <t>/products/magic-chef-model-hvdr1040b</t>
         </is>
       </c>
-      <c r="B173" s="3" t="inlineStr">
+      <c r="B173" t="inlineStr">
         <is>
           <t>Magic</t>
         </is>
       </c>
-      <c r="C173" s="3" t="inlineStr"/>
-      <c r="D173" s="3" t="inlineStr">
-        <is>
-          <t>Not processed yet</t>
-        </is>
-      </c>
-      <c r="E173" s="3" t="inlineStr"/>
-      <c r="F173" s="3" t="inlineStr"/>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Magic Chef 9.9 Cu. Ft. Top Freezer Refrigerator Black - HVDR1040B</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Model number - whole appliance</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>SERP (appliancefactoryparts, homedepot)</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="3" t="inlineStr">
@@ -5363,164 +5435,248 @@
       <c r="F174" s="3" t="inlineStr"/>
     </row>
     <row r="175">
-      <c r="A175" s="3" t="inlineStr">
+      <c r="A175" t="inlineStr">
         <is>
           <t>/products/midea-11002012040074</t>
         </is>
       </c>
-      <c r="B175" s="3" t="inlineStr">
+      <c r="B175" t="inlineStr">
         <is>
           <t>Midea</t>
         </is>
       </c>
-      <c r="C175" s="3" t="inlineStr"/>
-      <c r="D175" s="3" t="inlineStr">
-        <is>
-          <t>Not processed yet</t>
-        </is>
-      </c>
-      <c r="E175" s="3" t="inlineStr"/>
-      <c r="F175" s="3" t="inlineStr"/>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Midea Washer Single Phase Asynchronous Motor - 11002012040074</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr"/>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>encompass, hnkparts, searspartsdirect, genuinereplacementparts</t>
+        </is>
+      </c>
     </row>
     <row r="176">
-      <c r="A176" s="3" t="inlineStr">
+      <c r="A176" t="inlineStr">
         <is>
           <t>/products/panasonic-model-nnt945sfx</t>
         </is>
       </c>
-      <c r="B176" s="3" t="inlineStr">
+      <c r="B176" t="inlineStr">
         <is>
           <t>Panasonic</t>
         </is>
       </c>
-      <c r="C176" s="3" t="inlineStr"/>
-      <c r="D176" s="3" t="inlineStr">
-        <is>
-          <t>Not processed yet</t>
-        </is>
-      </c>
-      <c r="E176" s="3" t="inlineStr"/>
-      <c r="F176" s="3" t="inlineStr"/>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Panasonic 2.2 Cu. Ft. 1250W Inverter Countertop Microwave Stainless Steel - NN-T945SFX</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Model number - whole appliance</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>SERP (bjs, appliancefactoryparts)</t>
+        </is>
+      </c>
     </row>
     <row r="177">
-      <c r="A177" s="3" t="inlineStr">
+      <c r="A177" t="inlineStr">
         <is>
           <t>/products/powermate-a203120-power-tool-control-cable</t>
         </is>
       </c>
-      <c r="B177" s="3" t="inlineStr">
+      <c r="B177" t="inlineStr">
         <is>
           <t>Powermate</t>
         </is>
       </c>
-      <c r="C177" s="3" t="inlineStr"/>
-      <c r="D177" s="3" t="inlineStr">
-        <is>
-          <t>Not processed yet</t>
-        </is>
-      </c>
-      <c r="E177" s="3" t="inlineStr"/>
-      <c r="F177" s="3" t="inlineStr"/>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Powermate Tiller Forward Extension Control Cable - A203120</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr"/>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>ereplacementparts</t>
+        </is>
+      </c>
     </row>
     <row r="178">
-      <c r="A178" s="3" t="inlineStr">
+      <c r="A178" t="inlineStr">
         <is>
           <t>/products/ryobi-elect-tools-300627004</t>
         </is>
       </c>
-      <c r="B178" s="3" t="inlineStr">
+      <c r="B178" t="inlineStr">
         <is>
           <t>Ryobi</t>
         </is>
       </c>
-      <c r="C178" s="3" t="inlineStr"/>
-      <c r="D178" s="3" t="inlineStr">
-        <is>
-          <t>Not processed yet</t>
-        </is>
-      </c>
-      <c r="E178" s="3" t="inlineStr"/>
-      <c r="F178" s="3" t="inlineStr"/>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Ryobi Router 1/2" Collet Assembly - 300627004</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr"/>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>encompass, ereplacementparts, partswarehouse</t>
+        </is>
+      </c>
     </row>
     <row r="179">
-      <c r="A179" s="3" t="inlineStr">
+      <c r="A179" s="2" t="inlineStr">
         <is>
           <t>/products/whirlpool-model-caws923mq1</t>
         </is>
       </c>
-      <c r="B179" s="3" t="inlineStr">
+      <c r="B179" s="2" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="C179" s="3" t="inlineStr"/>
-      <c r="D179" s="3" t="inlineStr">
-        <is>
-          <t>Not processed yet</t>
-        </is>
-      </c>
-      <c r="E179" s="3" t="inlineStr"/>
-      <c r="F179" s="3" t="inlineStr"/>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>Whirlpool Top Load Washer - CAWS923MQ1</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>Model number - whole appliance, REVIEW</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>SERP (parts retailers list it as a washer model)</t>
+        </is>
+      </c>
     </row>
     <row r="180">
-      <c r="A180" s="3" t="inlineStr">
+      <c r="A180" t="inlineStr">
         <is>
           <t>/products/whirlpool-wp6-2011900</t>
         </is>
       </c>
-      <c r="B180" s="3" t="inlineStr">
+      <c r="B180" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="C180" s="3" t="inlineStr"/>
-      <c r="D180" s="3" t="inlineStr">
-        <is>
-          <t>Not processed yet</t>
-        </is>
-      </c>
-      <c r="E180" s="3" t="inlineStr"/>
-      <c r="F180" s="3" t="inlineStr"/>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Whirlpool Washer Brake Assembly - WP6-2011900</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Discontinued part</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>encompass, hnkparts, partsdr, applianceparts4all, appliancepartspros, searspartsdirect</t>
+        </is>
+      </c>
     </row>
     <row r="181">
-      <c r="A181" s="3" t="inlineStr">
+      <c r="A181" t="inlineStr">
         <is>
           <t>/products/ge-model-gtd75ecsl1ws</t>
         </is>
       </c>
-      <c r="B181" s="3" t="inlineStr">
+      <c r="B181" t="inlineStr">
         <is>
           <t>Ge</t>
         </is>
       </c>
-      <c r="C181" s="3" t="inlineStr"/>
-      <c r="D181" s="3" t="inlineStr">
-        <is>
-          <t>Not processed yet</t>
-        </is>
-      </c>
-      <c r="E181" s="3" t="inlineStr"/>
-      <c r="F181" s="3" t="inlineStr"/>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>GE 7.4 Cu. Ft. Smart Electric Dryer with HE Sensor Dry - GTD75ECSL1WS</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Model number - whole appliance</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>SERP (geappliances.com for GTD75ECSLWS, filtersfast)</t>
+        </is>
+      </c>
     </row>
     <row r="182">
-      <c r="A182" s="3" t="inlineStr">
+      <c r="A182" t="inlineStr">
         <is>
           <t>/products/lg-mgc66363126-dishwasher-control-panel</t>
         </is>
       </c>
-      <c r="B182" s="3" t="inlineStr">
+      <c r="B182" t="inlineStr">
         <is>
           <t>Lg</t>
         </is>
       </c>
-      <c r="C182" s="3" t="inlineStr"/>
-      <c r="D182" s="3" t="inlineStr">
-        <is>
-          <t>Not processed yet</t>
-        </is>
-      </c>
-      <c r="E182" s="3" t="inlineStr"/>
-      <c r="F182" s="3" t="inlineStr"/>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>LG WashTower Washer/Dryer Control Panel Assembly - MGC66363126</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Your URL says "dishwasher control panel" - competitors list it for LG WashTower models</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>shopjimmy, encompass, genuinereplacementparts</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="3" t="inlineStr">

</xml_diff>